<commit_message>
update for 24 sept
</commit_message>
<xml_diff>
--- a/12600637.xlsx
+++ b/12600637.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D01A918-7807-454D-97DD-88FDB9492621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A744121-D51A-46B0-A198-1DE4AE9177C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2914,24 +2914,44 @@
       <c r="N50" s="17"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+      <c r="A51" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B51" s="14">
+        <v>420</v>
+      </c>
+      <c r="C51" s="14">
+        <v>45</v>
+      </c>
+      <c r="D51" s="14">
+        <v>60</v>
+      </c>
+      <c r="E51" s="14">
+        <v>30</v>
+      </c>
+      <c r="F51" s="14">
+        <v>200</v>
+      </c>
+      <c r="G51" s="14">
+        <v>2</v>
+      </c>
+      <c r="H51" s="14">
+        <v>120</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>875</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
+        <v>565</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="M51" s="16"/>
       <c r="N51" s="17"/>
     </row>

</xml_diff>

<commit_message>
update for 25 sept
</commit_message>
<xml_diff>
--- a/12600637.xlsx
+++ b/12600637.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A744121-D51A-46B0-A198-1DE4AE9177C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BD24EF-8B33-45D0-A1B6-4247842E9DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2956,24 +2956,44 @@
       <c r="N51" s="17"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+      <c r="A52" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B52" s="14">
+        <v>420</v>
+      </c>
+      <c r="C52" s="14">
+        <v>45</v>
+      </c>
+      <c r="D52" s="14">
+        <v>100</v>
+      </c>
+      <c r="E52" s="14">
+        <v>45</v>
+      </c>
+      <c r="F52" s="14">
+        <v>300</v>
+      </c>
+      <c r="G52" s="14">
+        <v>5</v>
+      </c>
+      <c r="H52" s="14">
+        <v>100</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
+        <v>430</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="M52" s="16"/>
       <c r="N52" s="17"/>
     </row>

</xml_diff>

<commit_message>
update on 26 sept
</commit_message>
<xml_diff>
--- a/12600637.xlsx
+++ b/12600637.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BD24EF-8B33-45D0-A1B6-4247842E9DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C3A48F-8D99-4305-BF97-3E48E35CD08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Daily Log" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -353,7 +353,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -376,11 +376,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -420,6 +431,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -907,74 +921,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="21">
         <v>12600637</v>
       </c>
-      <c r="G2" s="20"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="20"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1198,6 +1212,9 @@
       <c r="A10" s="13">
         <v>46248</v>
       </c>
+      <c r="B10" s="18">
+        <v>420</v>
+      </c>
       <c r="C10" s="14">
         <v>0</v>
       </c>
@@ -1218,11 +1235,11 @@
       </c>
       <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v>450</v>
+        <v>870</v>
       </c>
       <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v>990</v>
+        <v>570</v>
       </c>
       <c r="K10" s="16" t="s">
         <v>49</v>
@@ -2998,24 +3015,44 @@
       <c r="N52" s="17"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+      <c r="A53" s="13">
+        <v>45926</v>
+      </c>
+      <c r="B53" s="14">
+        <v>540</v>
+      </c>
+      <c r="C53" s="14">
+        <v>45</v>
+      </c>
+      <c r="D53" s="14">
+        <v>100</v>
+      </c>
+      <c r="E53" s="14">
+        <v>60</v>
+      </c>
+      <c r="F53" s="14">
+        <v>0</v>
+      </c>
+      <c r="G53" s="14">
+        <v>0</v>
+      </c>
+      <c r="H53" s="14">
+        <v>100</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>845</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
+        <v>595</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="M53" s="16"/>
       <c r="N53" s="17"/>
     </row>

</xml_diff>

<commit_message>
update for 27 sept
</commit_message>
<xml_diff>
--- a/12600637.xlsx
+++ b/12600637.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C3A48F-8D99-4305-BF97-3E48E35CD08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A08D5C9-5377-44A7-BAF4-C999CDCFB1C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -242,6 +242,9 @@
   </si>
   <si>
     <t>low</t>
+  </si>
+  <si>
+    <t>bad</t>
   </si>
 </sst>
 </file>
@@ -3057,51 +3060,93 @@
       <c r="N53" s="17"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+      <c r="A54" s="13">
+        <v>45927</v>
+      </c>
+      <c r="B54" s="14">
+        <v>520</v>
+      </c>
+      <c r="C54" s="14">
+        <v>0</v>
+      </c>
+      <c r="D54" s="14">
+        <v>0</v>
+      </c>
+      <c r="E54" s="14">
+        <v>45</v>
+      </c>
+      <c r="F54" s="14">
+        <v>0</v>
+      </c>
+      <c r="G54" s="14">
+        <v>0</v>
+      </c>
+      <c r="H54" s="14">
+        <v>100</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>665</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
+        <v>775</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="M54" s="16"/>
       <c r="N54" s="17"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+      <c r="A55" s="13">
+        <v>45928</v>
+      </c>
+      <c r="B55" s="14">
+        <v>240</v>
+      </c>
+      <c r="C55" s="14">
+        <v>0</v>
+      </c>
+      <c r="D55" s="14">
+        <v>0</v>
+      </c>
+      <c r="E55" s="14">
+        <v>0</v>
+      </c>
+      <c r="F55" s="14">
+        <v>0</v>
+      </c>
+      <c r="G55" s="14">
+        <v>0</v>
+      </c>
+      <c r="H55" s="14">
+        <v>100</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>340</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
+        <v>1100</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="M55" s="16"/>
       <c r="N55" s="17"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="13"/>
+      <c r="A56" s="13">
+        <v>45929</v>
+      </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
       <c r="D56" s="14"/>
@@ -3118,7 +3163,9 @@
         <v/>
       </c>
       <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
+      <c r="L56" s="16" t="s">
+        <v>63</v>
+      </c>
       <c r="M56" s="16"/>
       <c r="N56" s="17"/>
     </row>

</xml_diff>

<commit_message>
update for 28,29,30  sept
</commit_message>
<xml_diff>
--- a/12600637.xlsx
+++ b/12600637.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satya\Desktop\datasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A08D5C9-5377-44A7-BAF4-C999CDCFB1C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B3D84B-BB7B-4E06-AA9F-3BF94A67A3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3147,22 +3147,38 @@
       <c r="A56" s="13">
         <v>45929</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
+      <c r="B56" s="14">
+        <v>240</v>
+      </c>
+      <c r="C56" s="14">
+        <v>0</v>
+      </c>
+      <c r="D56" s="14">
+        <v>0</v>
+      </c>
+      <c r="E56" s="14">
+        <v>0</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14">
+        <v>0</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
+        <v>240</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
+        <v>1200</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>69</v>
+      </c>
       <c r="L56" s="16" t="s">
         <v>63</v>
       </c>
@@ -3170,24 +3186,44 @@
       <c r="N56" s="17"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="13"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="15" t="str">
+      <c r="A57" s="13">
+        <v>45930</v>
+      </c>
+      <c r="B57" s="14">
+        <v>240</v>
+      </c>
+      <c r="C57" s="14">
+        <v>0</v>
+      </c>
+      <c r="D57" s="14">
+        <v>0</v>
+      </c>
+      <c r="E57" s="14">
+        <v>0</v>
+      </c>
+      <c r="F57" s="14">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14">
+        <v>0</v>
+      </c>
+      <c r="H57" s="14">
+        <v>0</v>
+      </c>
+      <c r="I57" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
+        <v>240</v>
+      </c>
+      <c r="J57" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
+        <v>1200</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>63</v>
+      </c>
       <c r="M57" s="16"/>
       <c r="N57" s="17"/>
     </row>

</xml_diff>